<commit_message>
Auto update P2P and organization activities 2026-09-08 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2189,7 +2189,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>"Píldores Aula Nucli (Yunier)
+11:30 - A nálisis de la Ecuación de Ventas</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>Yunier</t>
@@ -2240,7 +2245,8 @@
       <c r="C65" t="inlineStr">
         <is>
           <t>Presentacions Finals
-11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial</t>
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
+11:30 - Juan Carlos Morales: Biomecánica Ciclista</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-09 09:38
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2192,7 +2192,7 @@
       <c r="C63" t="inlineStr">
         <is>
           <t>"Píldores Aula Nucli (Yunier)
-11:30 - A nálisis de la Ecuación de Ventas</t>
+11:30 - Análisis de la Ecuación de Ventas</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Dago</t>
+          <t>11:00.- Incubadora de Projectes amb Dago</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2410,7 +2410,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>15:00-18:00 Zurich Day</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -2850,7 +2854,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Yunier</t>
+          <t>Saló de l'Ocupació</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2874,7 +2878,11 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Saló de l'Ocupació</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr">
         <is>
           <t>Dago</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-10 10:02
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2245,7 +2245,6 @@
       <c r="C65" t="inlineStr">
         <is>
           <t>Presentacions Finals
-11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
 11:30 - Juan Carlos Morales: Biomecánica Ciclista</t>
         </is>
       </c>
@@ -2356,7 +2355,13 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Presentacions Finals
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
+</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr">
         <is>
           <t>Dago</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-15 09:21
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2358,6 +2358,8 @@
       <c r="C69" t="inlineStr">
         <is>
           <t xml:space="preserve">Presentacions Finals
+10:00 - Violeta Correa: Gobernanza de Datos para la Red de Recarga Eléctrica de Barcelona
+10:30 - Francesca Pani: TBD
 11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
 </t>
         </is>
@@ -2417,7 +2419,8 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>15:00-18:00 Zurich Day</t>
+          <t>Time TBD: Explorando tu potencial a través del Cuadrante de Ofman
+15:00-18:00 Zurich Day</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-16 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2838,7 +2838,13 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Joan)
+10:00 - Sèries Temporals. Prediccions i explicabilitat.
+11:30 - Web Scraping amb Python</t>
+        </is>
+      </c>
       <c r="D87" t="inlineStr">
         <is>
           <t>Joan</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-16 09:33
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>"Píldores Aula Nucli (Yunier)
+          <t>Píldores Aula Nucli (Yunier)
 11:30 - Análisis de la Ecuación de Ventas</t>
         </is>
       </c>
@@ -2357,11 +2357,9 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Presentacions Finals
+          <t>Presentacions Finals
 10:00 - Violeta Correa: Gobernanza de Datos para la Red de Recarga Eléctrica de Barcelona
-10:30 - Francesca Pani: TBD
-11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
-</t>
+10:30 - Francesca Pani: TBD</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2419,8 +2417,9 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Time TBD: Explorando tu potencial a través del Cuadrante de Ofman
-15:00-18:00 Zurich Day</t>
+          <t>Píldores Aula Nucli (Irene)
+10:30 - Time TBD: Explorando tu potencial a través del Cuadrante de Ofman
+15:00 - 18:00 Zurich Day</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2688,7 +2687,13 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyectos:
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
+</t>
+        </is>
+      </c>
       <c r="D81" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-17 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2359,7 +2359,7 @@
         <is>
           <t>Presentacions Finals
 10:00 - Violeta Correa: Gobernanza de Datos para la Red de Recarga Eléctrica de Barcelona
-10:30 - Francesca Pani: TBD</t>
+10:30 - Francesca Pani: El pastel que no se reparte, Un retrato de la desigualdad, 1980-2024</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2531,7 +2531,7 @@
         <is>
           <t>Píldores Aula Nucli (Alana)
 Dinámica Grupal
-11:00 MVP: Producto mínimo viable</t>
+11:00 - Construcción de un MVP (Producto mínimo viable)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2639,7 +2639,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Píldores Aula Nucli (Dago)
+</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr">
         <is>
           <t>Dago</t>
@@ -2741,7 +2746,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Píldores Aula Nucli (Yunier)
+</t>
+        </is>
+      </c>
       <c r="D83" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-18 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2357,9 +2357,9 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Presentacions Finals
+          <t xml:space="preserve">Presentacions Finals
 10:00 - Violeta Correa: Gobernanza de Datos para la Red de Recarga Eléctrica de Barcelona
-10:30 - Francesca Pani: El pastel que no se reparte, Un retrato de la desigualdad, 1980-2024</t>
+</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2445,7 +2445,9 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Joan</t>
+          <t xml:space="preserve">Presentacions Finals
+10:30 - Francesca Pani: El pastel que no se reparte, Un retrato de la desigualdad, 1980-2024
+11:00 - Incubadora de Projectes amb Joan </t>
         </is>
       </c>
       <c r="D72" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-21 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2417,8 +2417,8 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Píldores Aula Nucli (Irene)
-10:30 - Time TBD: Explorando tu potencial a través del Cuadrante de Ofman
+          <t>Píldora Aula Nucli
+11:00 - 13:30 Taller de comunicación. Explorando la conciencia emocional y la comunicación no violenta para practicar cómo comunicarnos mejor y enfrentar conflictos en el contexto laboral y más allá. (Esto es un taller con prácticas en parejas y grupales, de una duración de dos horas y media, con una pequeña pausa en el medio.)
 15:00 - 18:00 Zurich Day</t>
         </is>
       </c>
@@ -2559,7 +2559,9 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Irene</t>
+          <t>Presentacions Finals
+10:30 - Jorge Aguilar Liévanos: TBD
+Incubadora de Projectes amb Irene</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2967,7 +2969,11 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Time TBD: Explorando tu potencial a través del Cuadrante de Ofman</t>
+        </is>
+      </c>
       <c r="D91" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-28 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3128,7 +3128,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
       <c r="D97" t="inlineStr">
         <is>
           <t>Joan</t>
@@ -3230,7 +3235,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
       <c r="D101" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -3332,7 +3342,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
       <c r="D105" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -3434,7 +3449,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>Dago</t>
@@ -3536,7 +3556,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
       <c r="D113" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-29 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2587,7 +2587,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Festivo</t>
+          <t>Dia sense assistència presencial a la ITAcademy</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2645,8 +2645,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Píldores Aula Nucli (Dago)
-</t>
+          <t>Pildores Aula Nucli (Dago) 11h                                                                                                                                                              Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-30 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2560,8 +2560,8 @@
       <c r="C76" t="inlineStr">
         <is>
           <t>Presentacions Finals
-10:30 - Jorge Aguilar Liévanos: TBD
-Incubadora de Projectes amb Irene</t>
+10:30 - Jorge Aguilar Liévanos: ¿Se está “apagando” el catalán? Lo que se dice y lo que dicen los datos.
+12:30 - Incubadora de Projectes amb Irene</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Pildores Aula Nucli (Dago) 11h                                                                                                                                                              Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
+          <t>Pildores Aula Nucli (Dago) 11h                                                                                                                                                                          Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-05 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2616,7 +2616,6 @@
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
 11:00 Alana 
-11:30 Joan 
 12:00 Yunier 
 12:30 Dago 
 13:00 Irene </t>
@@ -2645,7 +2644,8 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Pildores Aula Nucli (Dago) 11h                                                                                                                                                                          Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
+          <t>10:30 Weekly Joan
+Pildores Aula Nucli (Dago) 11h                                                                                                                                                                          Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-06 09:26
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2697,9 +2697,9 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proyectos:
+          <t>Proyectos:
 11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
-</t>
+11:30 - Biel Domènech-  FUTBOL: La possessió de la pilota està relacionada amb guanyar?</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-08 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2645,7 +2645,8 @@
       <c r="C79" t="inlineStr">
         <is>
           <t>10:30 Weekly Joan
-Pildores Aula Nucli (Dago) 11h                                                                                                                                                                          Cómo usar Typeform para hacer formularios y encuestas                                                                                                                                     Muchos de los reposotitorios de datos contienen errores debido a una mala contrucción de los formularios. El objetivo de esta píndola es adentrarnos a la construcción y creación de instrumentos de recoleccón de datos de forma cuantitativa. Aprenderás a hacer preguntas de acuerdo a su tipología: abiertas, cerrradas, de filtro, dicotómicas, multicotómicas, liker y de escala</t>
+Pildores Aula Nucli (Dago) 
+11h - Cómo usar Typeform para hacer formularios y encuestas</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2695,13 +2696,7 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Proyectos:
-11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
-11:30 - Biel Domènech-  FUTBOL: La possessió de la pilota està relacionada amb guanyar?</t>
-        </is>
-      </c>
+      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>Irene</t>
@@ -2802,7 +2797,14 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Proyectos:
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
+11:30 - Biel Domènech-  FUTBOL: La possessió de la pilota està relacionada amb guanyar?
+12:00 - Osley Sorio: Procesamiento local de informes medicos con Llama 3.2 3B</t>
+        </is>
+      </c>
       <c r="D85" t="inlineStr">
         <is>
           <t>Alana</t>
@@ -2970,7 +2972,8 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Time TBD: Explorando tu potencial a través del Cuadrante de Ofman</t>
+          <t>Píldores Aula Nucli (Irene)
+11 -Time TBD: Explorando tu potencial a través del Cuadrante de Ofman</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3400,7 +3403,12 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Joan)
+Machinne Learning</t>
+        </is>
+      </c>
       <c r="D107" t="inlineStr">
         <is>
           <t>Joan</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-15 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Saló de l'Ocupació</t>
+          <t>Incubadora de Projectes amb Yunier</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2914,7 +2914,8 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Saló de l'Ocupació</t>
+          <t>Proyectos:
+12:00 - Jorge Kundig: TBD</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-19 11:35
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3024,7 +3024,12 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Proyectos:
+10:30 - Leticia de Cuevillas: TBD</t>
+        </is>
+      </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-19 11:46
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3139,7 +3139,9 @@
       <c r="C97" t="inlineStr">
         <is>
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+Les presentacions es realitzaran a l'aula principal o en un altre espai.
+Proyectos:
+11:00 - Gina Caicedo Valencia: TBD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3465,7 +3467,9 @@
       <c r="C109" t="inlineStr">
         <is>
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+Les presentacions es realitzaran a l'aula principal o en un altre espai.
+Proyectos:
+11:00 - Desirée Diaz Risquete: TBD</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-20 09:35
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2861,8 +2861,7 @@
       <c r="C87" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Joan)
-10:00 - Sèries Temporals. Prediccions i explicabilitat.
-11:30 - Web Scraping amb Python</t>
+12:30 - 14:00 - Sèries Temporals. Prediccions i explicabilitat.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3027,7 +3026,8 @@
       <c r="C93" t="inlineStr">
         <is>
           <t>Proyectos:
-10:30 - Leticia de Cuevillas: TBD</t>
+10:30 - Leticia de Cuevillas: TBD
+12:00 - Irina Andrade: TBD</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-22 10:21
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2914,7 +2914,7 @@
       <c r="C89" t="inlineStr">
         <is>
           <t>Proyectos:
-12:00 - Jorge Kundig: TBD</t>
+12:00 - Jorge Kundig: Mengem Picant?</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3223,7 +3223,9 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Alana</t>
+          <t>Incubadora de Projectes amb Alana
+Proyectos:
+11:00 - Eloisa Estefania Thompson: TBD</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-23 09:20
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3143,7 +3143,11 @@
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.
 Proyectos:
-11:00 - Gina Caicedo Valencia: TBD</t>
+10:30 - Albert Armentano: TBD
+11:00 - Gina Caicedo Valencia: TBD
+11:30 - Natalia Cuenca: TBD
+12:00 - Alex Barbera Fabra: TBD
+12:30 - Cristina Fornaguera Torner: TBD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3167,7 +3171,106 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46336</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46337</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Alana
+Proyectos:
+11:00 - Eloisa Estefania Thompson: TBD</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>46338</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Presentación de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46342</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3178,105 +3281,103 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>46343</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="1" t="n">
-        <v>46336</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr">
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46344</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Dago</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="1" t="n">
-        <v>46337</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Alana
-Proyectos:
-11:00 - Eloisa Estefania Thompson: TBD</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr">
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
         <is>
           <t>Tutoría de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="1" t="n">
-        <v>46338</v>
-      </c>
-      <c r="B101" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>46345</v>
+      </c>
+      <c r="B105" t="inlineStr">
         <is>
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr">
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="1" t="n">
-        <v>46342</v>
-      </c>
-      <c r="B102" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46349</v>
+      </c>
+      <c r="B106" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3287,103 +3388,110 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>46350</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Joan)
+Machinne Learning</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="1" t="n">
-        <v>46343</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr">
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46351</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Yunier</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="1" t="n">
-        <v>46344</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Dago</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>46352</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.
+Proyectos:
+11:00 - Desirée Diaz Risquete: TBD</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
         <is>
           <t>Dago</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>46345</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr">
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>46349</v>
-      </c>
-      <c r="B106" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46356</v>
+      </c>
+      <c r="B110" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3394,110 +3502,103 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>46350</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Píldores Aula Nucli (Joan)
-Machinne Learning</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46358</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Joan</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="1" t="n">
-        <v>46351</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Yunier</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>46359</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
+Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
         <is>
           <t>Yunier</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>46352</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.
-Proyectos:
-11:00 - Desirée Diaz Risquete: TBD</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>46356</v>
-      </c>
-      <c r="B110" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>46370</v>
+      </c>
+      <c r="B114" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3508,103 +3609,103 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Dago</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Welcome / Weekley</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>46371</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Píldores Aula Nucli (Alana)
+11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>Alana</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr">
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Píldoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46372</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Incubadora de Projectes amb Irene</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
         <is>
           <t>Irene</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>46358</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Joan</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Tutoría de Proyectos</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>46373</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
         <is>
           <t>Joan</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="1" t="n">
-        <v>46359</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr">
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
         <is>
           <t>Presentación de Proyectos</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="1" t="n">
-        <v>46370</v>
-      </c>
-      <c r="B114" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46377</v>
+      </c>
+      <c r="B118" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t xml:space="preserve">Welcome: de 10:15 – 11:00 
 Weekly: 
@@ -3615,113 +3716,6 @@
 13:00 Irene </t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Dago</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>Welcome / Weekley</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="1" t="n">
-        <v>46371</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Martes</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Píldores Aula Nucli (Alana)
-11:00 - De la Teoria a la Pràctica: Apps amb Streamlit</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Píldoras</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="1" t="n">
-        <v>46372</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Miércoles</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Incubadora de Projectes amb Irene</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Tutoría de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="1" t="n">
-        <v>46373</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Jueves</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>Presentación de Proyectos</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="1" t="n">
-        <v>46377</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Lunes</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Welcome: de 10:15 – 11:00 
-Weekly: 
-11:00 Alana 
-11:30 Joan 
-12:00 Yunier 
-12:30 Dago 
-13:00 Irene </t>
-        </is>
-      </c>
       <c r="D118" t="inlineStr">
         <is>
           <t>Yunier</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-26 11:58
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2973,7 +2973,9 @@
       <c r="C91" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Irene)
-11 -Time TBD: Explorando tu potencial a través del Cuadrante de Ofman</t>
+10:30 - 13:45 (3 horas de taller, con una pausa de 15 minutos)
+Core Quadrant, el Cuadrante de las Cualidades Esenciales
+Explorando tus fortalezas y oportunidades de crecimiento a través del modelo de Daniel Ofman</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3412,7 +3414,8 @@
       <c r="C107" t="inlineStr">
         <is>
           <t>Píldores Aula Nucli (Joan)
-Machinne Learning</t>
+10:30 - Intro al Machine Learning
+12:00 - Intro al Web Scraping</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3761,7 +3764,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Incubadora de Projectes amb Alana</t>
+          <t>No Lectiu</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3785,7 +3788,11 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>No Lectiu</t>
+        </is>
+      </c>
       <c r="D121" t="inlineStr">
         <is>
           <t>Irene</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-27 09:41
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -2972,10 +2972,10 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Píldores Aula Nucli (Irene)
-10:30 - 13:45 (3 horas de taller, con una pausa de 15 minutos)
-Core Quadrant, el Cuadrante de las Cualidades Esenciales
-Explorando tus fortalezas y oportunidades de crecimiento a través del modelo de Daniel Ofman</t>
+          <t>Píldores Aula Nucli (Irene) - IN ENGLISH
+10:30–13:45 (3 hours of workshop, with a 15-minute break)
+Core Quadrant: The Quadrant of Core Qualities
+Exploring your strengths and developing your potential through Daniel Ofman’s model</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3028,9 +3028,8 @@
       <c r="C93" t="inlineStr">
         <is>
           <t>Proyectos:
-10:30 - Leticia de Cuevillas: TBD
 11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
-12:00 - Irina Andrade: TBD 
+11:30 - Irina Andrade: TBD 
 12:30 -Silvia Vilches: Segmentar para conquistar: Cómo perfilar clientes B2C con técnicas RFM y K-Means en las ventas flash del sector turísmo</t>
         </is>
       </c>
@@ -3145,11 +3144,13 @@
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.
 Proyectos:
-10:30 - Albert Armentano: TBD
+10:30 - Leticia de Cuevillas: TBD
 11:00 - Gina Caicedo Valencia: TBD
-11:30 - Natalia Cuenca: TBD
-12:00 - Alex Barbera Fabra: TBD
-12:30 - Cristina Fornaguera Torner: TBD</t>
+11:30 - Albert Armentano: TBD
+12:00 - Natalia Cuenca: TBD
+12:30 - Alex Barbera Fabra: TBD
+13:00 - Luis Rayón Liranzo: TBD
+13:30 - Leonardo Ruggiero: TBD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3248,7 +3249,8 @@
       <c r="C101" t="inlineStr">
         <is>
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
-Les presentacions es realitzaran a l'aula principal o en un altre espai.</t>
+Les presentacions es realitzaran a l'aula principal o en un altre espai.
+10:30 - Cristina Fornaguera Torner: TBD</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-28 09:59
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3028,8 +3028,7 @@
       <c r="C93" t="inlineStr">
         <is>
           <t>Proyectos:
-11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial
-11:30 - Irina Andrade: TBD 
+11:00 - Mariela Villca Vizalla: Análisis longitudinal y prospectivo de las profesiones frente al impacto de la inteligencia artificial 
 12:30 -Silvia Vilches: Segmentar para conquistar: Cómo perfilar clientes B2C con técnicas RFM y K-Means en las ventas flash del sector turísmo</t>
         </is>
       </c>
@@ -3148,7 +3147,7 @@
 11:00 - Gina Caicedo Valencia: TBD
 11:30 - Albert Armentano: TBD
 12:00 - Natalia Cuenca: TBD
-12:30 - Alex Barbera Fabra: TBD
+12:30 - Irina Andrade: TBD
 13:00 - Luis Rayón Liranzo: TBD
 13:30 - Leonardo Ruggiero: TBD</t>
         </is>
@@ -3250,7 +3249,8 @@
         <is>
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.
-10:30 - Cristina Fornaguera Torner: TBD</t>
+10:30 - Cristina Fornaguera Torner: TBD
+11:00 - Alex Barbera Fabra: TBD</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-29 09:32
</commit_message>
<xml_diff>
--- a/data/actividades.xlsx
+++ b/data/actividades.xlsx
@@ -3143,13 +3143,11 @@
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.
 Proyectos:
-10:30 - Leticia de Cuevillas: TBD
+10:30 - Leticia de Cuevillas: Composición y comportamiento de los títulos más prestados en las Bibliotecas Públicas de Madrid entre 2018 y 2026
 11:00 - Gina Caicedo Valencia: TBD
-11:30 - Albert Armentano: TBD
-12:00 - Natalia Cuenca: TBD
-12:30 - Irina Andrade: TBD
-13:00 - Luis Rayón Liranzo: TBD
-13:30 - Leonardo Ruggiero: TBD</t>
+11:30 -  Natalia Cuenca: TBD
+12:00 - Irina Andrade: TBD
+12:30 - Leonardo Ruggiero: TBD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3250,7 +3248,9 @@
           <t>Aula Reservada per a Activitats Alienes a la ITAcademy.
 Les presentacions es realitzaran a l'aula principal o en un altre espai.
 10:30 - Cristina Fornaguera Torner: TBD
-11:00 - Alex Barbera Fabra: TBD</t>
+11:00 - Alex Barbera Fabra: TBD
+11:30 - Luis Rayón Liranzo: TBD
+12:00 - Albert Armentano: TBD</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">

</xml_diff>